<commit_message>
Run: travel-timeline-2025.ts (Jan 6-7 corrected to NYC)
Alice confirmed flew Costa Rica → New York City on Jan 6.
Jan 6-7 updated from Unknown to New York.

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/data/travel-timeline-2025.xlsx
+++ b/data/travel-timeline-2025.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="404" uniqueCount="194">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="404" uniqueCount="192">
   <si>
     <t>2025 Travel Timeline — Substantial Presence Test</t>
   </si>
@@ -71,22 +71,16 @@
     <t>United States</t>
   </si>
   <si>
-    <t>medium</t>
-  </si>
-  <si>
-    <t>Flew back from Costa Rica on Jan 6. First confirmed US event NYC Jan 8.</t>
-  </si>
-  <si>
-    <t>City within US on Jan 6-7 unclear (likely Austin or NYC).</t>
+    <t>New York</t>
+  </si>
+  <si>
+    <t>Alice confirmed flew Costa Rica → NYC on Jan 6.</t>
   </si>
   <si>
     <t>2025-01-08</t>
   </si>
   <si>
     <t>2025-01-19</t>
-  </si>
-  <si>
-    <t>New York</t>
   </si>
   <si>
     <t>Confirmed events in NYC from Jan 8, including office day and various meetings.</t>
@@ -1172,33 +1166,33 @@
         <v>18</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E4" s="4">
         <v>2</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="G4" s="4" t="s">
         <v>20</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
     </row>
     <row r="5" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B5" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="B5" s="4" t="s">
-        <v>23</v>
-      </c>
       <c r="C5" s="4" t="s">
         <v>18</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="E5" s="4">
         <v>12</v>
@@ -1207,7 +1201,7 @@
         <v>13</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="H5" s="4" t="s">
         <v>15</v>
@@ -1215,16 +1209,16 @@
     </row>
     <row r="6" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C6" s="4" t="s">
         <v>18</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="E6" s="4">
         <v>1</v>
@@ -1233,7 +1227,7 @@
         <v>13</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="H6" s="4" t="s">
         <v>15</v>
@@ -1241,25 +1235,25 @@
     </row>
     <row r="7" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C7" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="D7" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="C7" s="5" t="s">
+      <c r="E7" s="5">
+        <v>18</v>
+      </c>
+      <c r="F7" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="G7" s="6" t="s">
         <v>30</v>
-      </c>
-      <c r="D7" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="E7" s="5">
-        <v>18</v>
-      </c>
-      <c r="F7" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="G7" s="6" t="s">
-        <v>32</v>
       </c>
       <c r="H7" s="6" t="s">
         <v>15</v>
@@ -1267,16 +1261,16 @@
     </row>
     <row r="8" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="C8" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="B8" s="7" t="s">
+      <c r="D8" s="7" t="s">
         <v>34</v>
-      </c>
-      <c r="C8" s="7" t="s">
-        <v>35</v>
-      </c>
-      <c r="D8" s="7" t="s">
-        <v>36</v>
       </c>
       <c r="E8" s="7">
         <v>6</v>
@@ -1285,7 +1279,7 @@
         <v>13</v>
       </c>
       <c r="G8" s="8" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="H8" s="8" t="s">
         <v>15</v>
@@ -1293,16 +1287,16 @@
     </row>
     <row r="9" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="7" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="E9" s="7">
         <v>1</v>
@@ -1311,7 +1305,7 @@
         <v>13</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="H9" s="8" t="s">
         <v>15</v>
@@ -1319,25 +1313,25 @@
     </row>
     <row r="10" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="B10" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="C10" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="B10" s="9" t="s">
+      <c r="D10" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="C10" s="9" t="s">
+      <c r="E10" s="9">
+        <v>13</v>
+      </c>
+      <c r="F10" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G10" s="10" t="s">
         <v>42</v>
-      </c>
-      <c r="D10" s="9" t="s">
-        <v>43</v>
-      </c>
-      <c r="E10" s="9">
-        <v>13</v>
-      </c>
-      <c r="F10" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G10" s="10" t="s">
-        <v>44</v>
       </c>
       <c r="H10" s="10" t="s">
         <v>15</v>
@@ -1345,16 +1339,16 @@
     </row>
     <row r="11" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C11" s="4" t="s">
         <v>18</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="E11" s="4">
         <v>1</v>
@@ -1363,7 +1357,7 @@
         <v>13</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="H11" s="4" t="s">
         <v>15</v>
@@ -1371,16 +1365,16 @@
     </row>
     <row r="12" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C12" s="4" t="s">
         <v>18</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="E12" s="4">
         <v>7</v>
@@ -1389,7 +1383,7 @@
         <v>13</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="H12" s="4" t="s">
         <v>15</v>
@@ -1397,16 +1391,16 @@
     </row>
     <row r="13" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="D13" s="4" t="s">
         <v>50</v>
-      </c>
-      <c r="B13" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="C13" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="D13" s="4" t="s">
-        <v>52</v>
       </c>
       <c r="E13" s="4">
         <v>11</v>
@@ -1415,7 +1409,7 @@
         <v>13</v>
       </c>
       <c r="G13" s="4" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="H13" s="4" t="s">
         <v>15</v>
@@ -1423,25 +1417,25 @@
     </row>
     <row r="14" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="E14" s="4">
+        <v>15</v>
+      </c>
+      <c r="F14" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G14" s="4" t="s">
         <v>54</v>
-      </c>
-      <c r="B14" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="C14" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="D14" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="E14" s="4">
-        <v>15</v>
-      </c>
-      <c r="F14" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="G14" s="4" t="s">
-        <v>56</v>
       </c>
       <c r="H14" s="4" t="s">
         <v>15</v>
@@ -1449,16 +1443,16 @@
     </row>
     <row r="15" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="4" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="C15" s="4" t="s">
         <v>18</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="E15" s="4">
         <v>1</v>
@@ -1467,7 +1461,7 @@
         <v>13</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="H15" s="4" t="s">
         <v>15</v>
@@ -1475,16 +1469,16 @@
     </row>
     <row r="16" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="B16" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C16" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="B16" s="9" t="s">
+      <c r="D16" s="9" t="s">
         <v>60</v>
-      </c>
-      <c r="C16" s="9" t="s">
-        <v>61</v>
-      </c>
-      <c r="D16" s="9" t="s">
-        <v>62</v>
       </c>
       <c r="E16" s="9">
         <v>10</v>
@@ -1493,7 +1487,7 @@
         <v>13</v>
       </c>
       <c r="G16" s="10" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="H16" s="10" t="s">
         <v>15</v>
@@ -1501,16 +1495,16 @@
     </row>
     <row r="17" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" s="4" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="C17" s="4" t="s">
         <v>18</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="E17" s="4">
         <v>11</v>
@@ -1519,7 +1513,7 @@
         <v>13</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="H17" s="4" t="s">
         <v>15</v>
@@ -1527,16 +1521,16 @@
     </row>
     <row r="18" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" s="4" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="C18" s="4" t="s">
         <v>18</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E18" s="4">
         <v>7</v>
@@ -1545,7 +1539,7 @@
         <v>13</v>
       </c>
       <c r="G18" s="4" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="H18" s="4" t="s">
         <v>15</v>
@@ -1553,16 +1547,16 @@
     </row>
     <row r="19" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" s="4" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="C19" s="4" t="s">
         <v>18</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E19" s="4">
         <v>1</v>
@@ -1571,7 +1565,7 @@
         <v>13</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="H19" s="4" t="s">
         <v>15</v>
@@ -1579,16 +1573,16 @@
     </row>
     <row r="20" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" s="7" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="C20" s="7" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="D20" s="7" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="E20" s="7">
         <v>23</v>
@@ -1597,7 +1591,7 @@
         <v>13</v>
       </c>
       <c r="G20" s="8" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H20" s="8" t="s">
         <v>15</v>
@@ -1605,16 +1599,16 @@
     </row>
     <row r="21" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" s="4" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="C21" s="4" t="s">
         <v>18</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E21" s="4">
         <v>5</v>
@@ -1623,7 +1617,7 @@
         <v>13</v>
       </c>
       <c r="G21" s="4" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="H21" s="4" t="s">
         <v>15</v>
@@ -1631,16 +1625,16 @@
     </row>
     <row r="22" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="D22" s="4" t="s">
         <v>77</v>
-      </c>
-      <c r="B22" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="C22" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="D22" s="4" t="s">
-        <v>79</v>
       </c>
       <c r="E22" s="4">
         <v>9</v>
@@ -1649,7 +1643,7 @@
         <v>13</v>
       </c>
       <c r="G22" s="4" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="H22" s="4" t="s">
         <v>15</v>
@@ -1657,16 +1651,16 @@
     </row>
     <row r="23" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" s="4" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="C23" s="4" t="s">
         <v>18</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E23" s="4">
         <v>1</v>
@@ -1675,7 +1669,7 @@
         <v>13</v>
       </c>
       <c r="G23" s="4" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="H23" s="4" t="s">
         <v>15</v>
@@ -1683,16 +1677,16 @@
     </row>
     <row r="24" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" s="11" t="s">
+        <v>81</v>
+      </c>
+      <c r="B24" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="C24" s="11" t="s">
         <v>83</v>
       </c>
-      <c r="B24" s="11" t="s">
+      <c r="D24" s="11" t="s">
         <v>84</v>
-      </c>
-      <c r="C24" s="11" t="s">
-        <v>85</v>
-      </c>
-      <c r="D24" s="11" t="s">
-        <v>86</v>
       </c>
       <c r="E24" s="11">
         <v>6</v>
@@ -1701,7 +1695,7 @@
         <v>13</v>
       </c>
       <c r="G24" s="12" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="H24" s="12" t="s">
         <v>15</v>
@@ -1709,16 +1703,16 @@
     </row>
     <row r="25" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="B25" s="13" t="s">
+        <v>87</v>
+      </c>
+      <c r="C25" s="13" t="s">
         <v>88</v>
       </c>
-      <c r="B25" s="13" t="s">
+      <c r="D25" s="13" t="s">
         <v>89</v>
-      </c>
-      <c r="C25" s="13" t="s">
-        <v>90</v>
-      </c>
-      <c r="D25" s="13" t="s">
-        <v>91</v>
       </c>
       <c r="E25" s="13">
         <v>11</v>
@@ -1727,7 +1721,7 @@
         <v>13</v>
       </c>
       <c r="G25" s="14" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="H25" s="14" t="s">
         <v>15</v>
@@ -1735,16 +1729,16 @@
     </row>
     <row r="26" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" s="7" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="B26" s="7" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C26" s="7" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="D26" s="7" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="E26" s="7">
         <v>4</v>
@@ -1753,7 +1747,7 @@
         <v>13</v>
       </c>
       <c r="G26" s="8" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H26" s="8" t="s">
         <v>15</v>
@@ -1761,16 +1755,16 @@
     </row>
     <row r="27" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" s="4" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="C27" s="4" t="s">
         <v>18</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E27" s="4">
         <v>7</v>
@@ -1779,7 +1773,7 @@
         <v>13</v>
       </c>
       <c r="G27" s="4" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="H27" s="4" t="s">
         <v>15</v>
@@ -1787,16 +1781,16 @@
     </row>
     <row r="28" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="B28" s="9" t="s">
+        <v>97</v>
+      </c>
+      <c r="C28" s="9" t="s">
         <v>98</v>
       </c>
-      <c r="B28" s="9" t="s">
+      <c r="D28" s="9" t="s">
         <v>99</v>
-      </c>
-      <c r="C28" s="9" t="s">
-        <v>100</v>
-      </c>
-      <c r="D28" s="9" t="s">
-        <v>101</v>
       </c>
       <c r="E28" s="9">
         <v>4</v>
@@ -1805,7 +1799,7 @@
         <v>13</v>
       </c>
       <c r="G28" s="10" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="H28" s="10" t="s">
         <v>15</v>
@@ -1813,10 +1807,10 @@
     </row>
     <row r="29" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29" s="9" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="B29" s="9" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="C29" s="9" t="s">
         <v>11</v>
@@ -1831,7 +1825,7 @@
         <v>13</v>
       </c>
       <c r="G29" s="10" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="H29" s="10" t="s">
         <v>15</v>
@@ -1839,16 +1833,16 @@
     </row>
     <row r="30" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" s="4" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C30" s="4" t="s">
         <v>18</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E30" s="4">
         <v>9</v>
@@ -1857,7 +1851,7 @@
         <v>13</v>
       </c>
       <c r="G30" s="4" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="H30" s="4" t="s">
         <v>15</v>
@@ -1865,16 +1859,16 @@
     </row>
     <row r="31" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" s="4" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="C31" s="4" t="s">
         <v>18</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="E31" s="4">
         <v>5</v>
@@ -1883,7 +1877,7 @@
         <v>13</v>
       </c>
       <c r="G31" s="4" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="H31" s="4" t="s">
         <v>15</v>
@@ -1891,16 +1885,16 @@
     </row>
     <row r="32" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" s="4" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="C32" s="4" t="s">
         <v>18</v>
       </c>
       <c r="D32" s="4" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E32" s="4">
         <v>4</v>
@@ -1909,7 +1903,7 @@
         <v>13</v>
       </c>
       <c r="G32" s="4" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="H32" s="4" t="s">
         <v>15</v>
@@ -1917,16 +1911,16 @@
     </row>
     <row r="33" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" s="7" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="B33" s="7" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="C33" s="7" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="D33" s="7" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="E33" s="7">
         <v>13</v>
@@ -1935,7 +1929,7 @@
         <v>13</v>
       </c>
       <c r="G33" s="8" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H33" s="8" t="s">
         <v>15</v>
@@ -1943,16 +1937,16 @@
     </row>
     <row r="34" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" s="13" t="s">
+        <v>115</v>
+      </c>
+      <c r="B34" s="13" t="s">
+        <v>116</v>
+      </c>
+      <c r="C34" s="13" t="s">
+        <v>88</v>
+      </c>
+      <c r="D34" s="13" t="s">
         <v>117</v>
-      </c>
-      <c r="B34" s="13" t="s">
-        <v>118</v>
-      </c>
-      <c r="C34" s="13" t="s">
-        <v>90</v>
-      </c>
-      <c r="D34" s="13" t="s">
-        <v>119</v>
       </c>
       <c r="E34" s="13">
         <v>9</v>
@@ -1961,7 +1955,7 @@
         <v>13</v>
       </c>
       <c r="G34" s="14" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="H34" s="14" t="s">
         <v>15</v>
@@ -1969,16 +1963,16 @@
     </row>
     <row r="35" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35" s="13" t="s">
+        <v>118</v>
+      </c>
+      <c r="B35" s="13" t="s">
+        <v>119</v>
+      </c>
+      <c r="C35" s="13" t="s">
+        <v>88</v>
+      </c>
+      <c r="D35" s="13" t="s">
         <v>120</v>
-      </c>
-      <c r="B35" s="13" t="s">
-        <v>121</v>
-      </c>
-      <c r="C35" s="13" t="s">
-        <v>90</v>
-      </c>
-      <c r="D35" s="13" t="s">
-        <v>122</v>
       </c>
       <c r="E35" s="13">
         <v>2</v>
@@ -1987,7 +1981,7 @@
         <v>13</v>
       </c>
       <c r="G35" s="14" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="H35" s="14" t="s">
         <v>15</v>
@@ -1995,16 +1989,16 @@
     </row>
     <row r="36" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36" s="11" t="s">
+        <v>122</v>
+      </c>
+      <c r="B36" s="11" t="s">
+        <v>123</v>
+      </c>
+      <c r="C36" s="11" t="s">
+        <v>83</v>
+      </c>
+      <c r="D36" s="11" t="s">
         <v>124</v>
-      </c>
-      <c r="B36" s="11" t="s">
-        <v>125</v>
-      </c>
-      <c r="C36" s="11" t="s">
-        <v>85</v>
-      </c>
-      <c r="D36" s="11" t="s">
-        <v>126</v>
       </c>
       <c r="E36" s="11">
         <v>10</v>
@@ -2013,7 +2007,7 @@
         <v>13</v>
       </c>
       <c r="G36" s="12" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="H36" s="12" t="s">
         <v>15</v>
@@ -2021,16 +2015,16 @@
     </row>
     <row r="37" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37" s="7" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B37" s="7" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="C37" s="7" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="D37" s="7" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="E37" s="7">
         <v>11</v>
@@ -2039,7 +2033,7 @@
         <v>13</v>
       </c>
       <c r="G37" s="8" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H37" s="8" t="s">
         <v>15</v>
@@ -2047,16 +2041,16 @@
     </row>
     <row r="38" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38" s="4" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="B38" s="4" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="C38" s="4" t="s">
         <v>18</v>
       </c>
       <c r="D38" s="4" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E38" s="4">
         <v>10</v>
@@ -2065,7 +2059,7 @@
         <v>13</v>
       </c>
       <c r="G38" s="4" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="H38" s="4" t="s">
         <v>15</v>
@@ -2073,16 +2067,16 @@
     </row>
     <row r="39" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39" s="4" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="B39" s="4" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="C39" s="4" t="s">
         <v>18</v>
       </c>
       <c r="D39" s="4" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="E39" s="4">
         <v>2</v>
@@ -2091,7 +2085,7 @@
         <v>13</v>
       </c>
       <c r="G39" s="4" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="H39" s="4" t="s">
         <v>15</v>
@@ -2099,16 +2093,16 @@
     </row>
     <row r="40" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40" s="4" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="B40" s="4" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="C40" s="4" t="s">
         <v>18</v>
       </c>
       <c r="D40" s="4" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="E40" s="4">
         <v>1</v>
@@ -2117,24 +2111,24 @@
         <v>13</v>
       </c>
       <c r="G40" s="4" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="H40" s="4" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="41" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A41" s="4" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="B41" s="4" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="C41" s="4" t="s">
         <v>18</v>
       </c>
       <c r="D41" s="4" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E41" s="4">
         <v>14</v>
@@ -2143,7 +2137,7 @@
         <v>13</v>
       </c>
       <c r="G41" s="4" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="H41" s="4" t="s">
         <v>15</v>
@@ -2151,16 +2145,16 @@
     </row>
     <row r="42" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A42" s="4" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="B42" s="4" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="C42" s="4" t="s">
         <v>18</v>
       </c>
       <c r="D42" s="4" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="E42" s="4">
         <v>8</v>
@@ -2169,7 +2163,7 @@
         <v>13</v>
       </c>
       <c r="G42" s="4" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="H42" s="4" t="s">
         <v>15</v>
@@ -2177,16 +2171,16 @@
     </row>
     <row r="43" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A43" s="4" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="B43" s="4" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="C43" s="4" t="s">
         <v>18</v>
       </c>
       <c r="D43" s="4" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E43" s="4">
         <v>25</v>
@@ -2195,7 +2189,7 @@
         <v>13</v>
       </c>
       <c r="G43" s="4" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="H43" s="4" t="s">
         <v>15</v>
@@ -2203,16 +2197,16 @@
     </row>
     <row r="44" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A44" s="9" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="B44" s="9" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="C44" s="9" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D44" s="9" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="E44" s="9">
         <v>3</v>
@@ -2221,7 +2215,7 @@
         <v>13</v>
       </c>
       <c r="G44" s="10" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="H44" s="10" t="s">
         <v>15</v>
@@ -2229,16 +2223,16 @@
     </row>
     <row r="45" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A45" s="4" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="B45" s="4" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="C45" s="4" t="s">
         <v>18</v>
       </c>
       <c r="D45" s="4" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="E45" s="4">
         <v>7</v>
@@ -2247,7 +2241,7 @@
         <v>13</v>
       </c>
       <c r="G45" s="4" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="H45" s="4" t="s">
         <v>15</v>
@@ -2255,16 +2249,16 @@
     </row>
     <row r="46" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A46" s="4" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="B46" s="4" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="C46" s="4" t="s">
         <v>18</v>
       </c>
       <c r="D46" s="4" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E46" s="4">
         <v>7</v>
@@ -2273,7 +2267,7 @@
         <v>13</v>
       </c>
       <c r="G46" s="4" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="H46" s="4" t="s">
         <v>15</v>
@@ -2281,16 +2275,16 @@
     </row>
     <row r="47" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A47" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="B47" s="4" t="s">
+        <v>153</v>
+      </c>
+      <c r="C47" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="D47" s="4" t="s">
         <v>154</v>
-      </c>
-      <c r="B47" s="4" t="s">
-        <v>155</v>
-      </c>
-      <c r="C47" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="D47" s="4" t="s">
-        <v>156</v>
       </c>
       <c r="E47" s="4">
         <v>5</v>
@@ -2299,7 +2293,7 @@
         <v>13</v>
       </c>
       <c r="G47" s="4" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="H47" s="4" t="s">
         <v>15</v>
@@ -2307,16 +2301,16 @@
     </row>
     <row r="48" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A48" s="4" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="B48" s="4" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="C48" s="4" t="s">
         <v>18</v>
       </c>
       <c r="D48" s="4" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E48" s="4">
         <v>5</v>
@@ -2325,7 +2319,7 @@
         <v>13</v>
       </c>
       <c r="G48" s="4" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="H48" s="4" t="s">
         <v>15</v>
@@ -2333,16 +2327,16 @@
     </row>
     <row r="49" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A49" s="7" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="B49" s="7" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="C49" s="7" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="D49" s="7" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="E49" s="7">
         <v>8</v>
@@ -2351,7 +2345,7 @@
         <v>13</v>
       </c>
       <c r="G49" s="8" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H49" s="8" t="s">
         <v>15</v>
@@ -2359,16 +2353,16 @@
     </row>
     <row r="50" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A50" s="7" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="B50" s="7" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="C50" s="7" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="D50" s="7" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="E50" s="7">
         <v>1</v>
@@ -2377,7 +2371,7 @@
         <v>13</v>
       </c>
       <c r="G50" s="8" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="H50" s="8" t="s">
         <v>15</v>
@@ -2385,16 +2379,16 @@
     </row>
     <row r="51" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A51" s="9" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="B51" s="9" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="C51" s="9" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="D51" s="9" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="E51" s="9">
         <v>1</v>
@@ -2403,7 +2397,7 @@
         <v>13</v>
       </c>
       <c r="G51" s="10" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="H51" s="10" t="s">
         <v>15</v>
@@ -2411,16 +2405,16 @@
     </row>
     <row r="52" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A52" s="9" t="s">
+        <v>166</v>
+      </c>
+      <c r="B52" s="9" t="s">
+        <v>167</v>
+      </c>
+      <c r="C52" s="9" t="s">
         <v>168</v>
       </c>
-      <c r="B52" s="9" t="s">
+      <c r="D52" s="9" t="s">
         <v>169</v>
-      </c>
-      <c r="C52" s="9" t="s">
-        <v>170</v>
-      </c>
-      <c r="D52" s="9" t="s">
-        <v>171</v>
       </c>
       <c r="E52" s="9">
         <v>4</v>
@@ -2429,7 +2423,7 @@
         <v>13</v>
       </c>
       <c r="G52" s="10" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="H52" s="10" t="s">
         <v>15</v>
@@ -2437,7 +2431,7 @@
     </row>
     <row r="54" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A54" s="15" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.25">
@@ -2445,55 +2439,55 @@
         <v>18</v>
       </c>
       <c r="B55" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
     </row>
     <row r="56" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A56" s="16" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B56" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
     </row>
     <row r="57" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A57" s="16" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="B57" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
     </row>
     <row r="58" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A58" s="16" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B58" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
     </row>
     <row r="59" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A59" s="16" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B59" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
     </row>
     <row r="60" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A60" s="16" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B60" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
     </row>
     <row r="61" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A61" s="16" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B61" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
     </row>
     <row r="62" spans="1:2" x14ac:dyDescent="0.25">
@@ -2501,47 +2495,47 @@
         <v>11</v>
       </c>
       <c r="B62" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
     </row>
     <row r="63" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A63" s="16" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="B63" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
     </row>
     <row r="64" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A64" s="16" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="B64" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
     </row>
     <row r="65" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A65" s="16" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="B65" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
     </row>
     <row r="66" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A66" s="16" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="B66" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
     </row>
     <row r="68" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A68" s="17" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="B68" s="18" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="C68" s="18"/>
       <c r="D68" s="18"/>
@@ -2552,10 +2546,10 @@
     </row>
     <row r="69" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A69" s="19" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="B69" s="18" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="C69" s="18"/>
       <c r="D69" s="18"/>
@@ -2589,7 +2583,7 @@
         <v>3</v>
       </c>
       <c r="B1" s="20" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
@@ -2602,7 +2596,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B3">
         <v>67</v>
@@ -2610,7 +2604,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="B4">
         <v>22</v>
@@ -2618,7 +2612,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B5">
         <v>18</v>
@@ -2626,7 +2620,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B6">
         <v>16</v>
@@ -2634,7 +2628,7 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B7">
         <v>13</v>
@@ -2642,7 +2636,7 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B8">
         <v>10</v>
@@ -2658,7 +2652,7 @@
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="B10">
         <v>13</v>
@@ -2666,7 +2660,7 @@
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="B11">
         <v>7</v>
@@ -2674,7 +2668,7 @@
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="B12">
         <v>4</v>
@@ -2682,7 +2676,7 @@
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="B13">
         <v>1</v>
@@ -2690,10 +2684,10 @@
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="B15" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
     </row>
   </sheetData>

</xml_diff>